<commit_message>
test(responsive): them Playwright that + fix build da trang + checklist demo
- them playwright.config.ts + tests/responsive.spec.ts: 15 trang x 5 moc (360/480/768/1024/1280) khong tran ngang + menu mobile (77 PASS)

- sua selector ready hero-detail/items; dong bo test-hero-admin voi hero-admin.html dung khung quan tri chung (16/16 file mini-DOM PASS)

- vite.config.js: build multi-page du 16 trang, chep src/js + src/data vao dist

- responsive: common.css (account-area 480px) + compare.css (@media 480px)

- README muc 6: Checklist kiem thu & demo; cap nhat aov-hub-data.json + AOV_HUB.xlsx (STT 48/49/50 da xong)
</commit_message>
<xml_diff>
--- a/AOV_HUB.xlsx
+++ b/AOV_HUB.xlsx
@@ -257,11 +257,11 @@
         </is>
       </c>
       <c r="B8" s="2">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">index.html + 14 trang trong src/pages.</t>
+          <t xml:space="preserve">index.html + 15 trang trong src/pages.</t>
         </is>
       </c>
     </row>
@@ -287,7 +287,7 @@
         </is>
       </c>
       <c r="B10" s="2">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -303,147 +303,181 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">15/15 file PASS</t>
+          <t xml:space="preserve">16/16 file PASS + 77 E2E PASS</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">687 kiểm tra PASS, 0 FAIL (mini-DOM, chưa chạy trình duyệt thật).</t>
+          <t xml:space="preserve">mini-DOM: 16 file PASS; Playwright (trình duyệt thật): 77 PASS.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Công việc chính hoàn thành</t>
-        </is>
-      </c>
-      <c r="B12" s="2">
-        <v>41</v>
+          <t xml:space="preserve">Responsive (trình duyệt thật)</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">77/77 PASS</t>
+        </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">STT 1-50, xem sheet 'Công việc chính'.</t>
+          <t xml:space="preserve">15 trang × 360/480/768/1024/1280 không tràn ngang; menu mobile hoạt động.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Công việc chính làm một phần</t>
-        </is>
-      </c>
-      <c r="B13" s="2">
-        <v>9</v>
+          <t xml:space="preserve">Đóng gói (npm run build)</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">16/16 trang</t>
+        </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">STT 6,13,18,20,29,36,48,49,50.</t>
+          <t xml:space="preserve">vite.config.js cấu hình multi-page; chép src/js + src/data vào dist; kiểm tra bằng npm run preview.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Công việc chính chưa làm</t>
+          <t xml:space="preserve">Công việc chính hoàn thành</t>
         </is>
       </c>
       <c r="B14" s="2">
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Không còn mục nào ở mức chưa làm trong 50 việc chính.</t>
+          <t xml:space="preserve">STT 1-50; các mục 48, 49, 50 nay đã xong.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lỗi đã xử lý trong lần review</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">L14, L15, L17, L18, L23, L24</t>
-        </is>
+          <t xml:space="preserve">Công việc chính làm một phần</t>
+        </is>
+      </c>
+      <c r="B15" s="2">
+        <v>6</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">open redirect, băm mật khẩu, backup.rar, README, trang 404, responsive admin.</t>
+          <t xml:space="preserve">STT 6,13,18,20,29,36.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lỗi còn tồn</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">L06, L12, L19, L20, L22</t>
-        </is>
+          <t xml:space="preserve">Công việc chính chưa làm</t>
+        </is>
+      </c>
+      <c r="B16" s="2">
+        <v>0</v>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">lane/title, build còn thiếu, tách profile.js, header search, tiêu chí nổi bật.</t>
+          <t xml:space="preserve">Không còn mục nào ở mức chưa làm trong 50 việc chính.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kế hoạch mở rộng đã xong</t>
+          <t xml:space="preserve">Lỗi đã xử lý trong lần review</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">CM02, KD01, KD02, AD01-AD04, AD10</t>
+          <t xml:space="preserve">L14, L15, L17, L18, L23, L24</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nhật ký admin, trạng thái bài, duyệt trước, quản lý tướng CRUD.</t>
+          <t xml:space="preserve">open redirect, băm mật khẩu, backup.rar, README, trang 404, responsive admin.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kế hoạch mở rộng kế tiếp</t>
+          <t xml:space="preserve">Lỗi còn tồn</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KD03, AD05-AD09, HD01-HD10</t>
+          <t xml:space="preserve">L06, L12, L19, L20, L22</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Duyệt/từ chối bài, quản lý trang bị/build, hướng dẫn build.</t>
+          <t xml:space="preserve">lane/title, build còn thiếu, tách profile.js, header search, tiêu chí nổi bật.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">Kế hoạch mở rộng đã xong</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CM02, KD01, KD02, AD01-AD04, AD10</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nhật ký admin, trạng thái bài, duyệt trước, quản lý tướng CRUD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kế hoạch mở rộng kế tiếp</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KD03, AD05-AD09, HD01-HD10</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Duyệt/từ chối bài, quản lý trang bị/build, hướng dẫn build.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">Rủi ro chính</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Không backend; quyền admin chỉ ở trình duyệt</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Dữ liệu nằm ở JSON/LocalStorage/File System Access; lớp clean architecture chưa được nạp; test chưa chạy trên trình duyệt thật.</t>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dữ liệu nằm ở JSON/LocalStorage/File System Access; lớp clean architecture chưa được nạp; đã có test Playwright trên trình duyệt thật (77 PASS) nhưng vẫn chỉ là demo, không phải bảo mật thật.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C19"/>
+  <autoFilter ref="A1:C21"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1727,9 +1761,9 @@
           <t xml:space="preserve">Responsive: trang chủ, danh sách/chi tiết tướng/trang bị</t>
         </is>
       </c>
-      <c r="C49" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Một phần</t>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã xong</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
@@ -1739,12 +1773,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">hero/home/item/build/favorite/compare/admin đều có @media.</t>
-        </is>
-      </c>
-      <c r="G49" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Kiểm tra trên thiết bị thật.</t>
+          <t xml:space="preserve">hero/home/item/build/favorite/compare/admin đều có @media; Playwright xác nhận 15 trang × 5 mốc không tràn ngang.</t>
         </is>
       </c>
     </row>
@@ -1757,9 +1786,9 @@
           <t xml:space="preserve">Responsive: Feed, chi tiết bài viết, form Account</t>
         </is>
       </c>
-      <c r="C50" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Một phần</t>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã xong</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -1769,12 +1798,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">feed.css (5 @media), common.css (5), auth.css (2).</t>
-        </is>
-      </c>
-      <c r="G50" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Kiểm tra trên thiết bị thật.</t>
+          <t xml:space="preserve">feed.css (5 @media), common.css (5), auth.css (2); kiểm tra thật ở 360/480/768/1024/1280.</t>
         </is>
       </c>
     </row>
@@ -1787,9 +1811,9 @@
           <t xml:space="preserve">Checklist test, fix lỗi, chuẩn bị demo</t>
         </is>
       </c>
-      <c r="C51" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Một phần</t>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã xong</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
@@ -1799,12 +1823,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">15 file test PASS, 687 kiểm tra, 0 FAIL (mini-DOM).</t>
-        </is>
-      </c>
-      <c r="G51" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Thêm test trình duyệt thật; lập checklist demo.</t>
+          <t xml:space="preserve">16 file test mini-DOM PASS; 77 test Playwright PASS; build 16 trang; checklist demo ở README (mục 6).</t>
         </is>
       </c>
     </row>
@@ -4471,7 +4490,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bộ test tự động (tools/)</t>
+          <t xml:space="preserve">Bộ test tự động (tools/ + tests/)</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -4481,7 +4500,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">15 file test PASS, 687 kiểm tra PASS, 0 FAIL (mini-DOM).</t>
+          <t xml:space="preserve">16 file test mini-DOM PASS; 77 test Playwright responsive PASS (trình duyệt thật).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(excel): cap nhat AOV_HUB.xlsx theo trang thai code moi nhat
</commit_message>
<xml_diff>
--- a/AOV_HUB.xlsx
+++ b/AOV_HUB.xlsx
@@ -15,6 +15,7 @@
     <sheet name="Việc nên làm tiếp" sheetId="7" r:id="rId7"/>
     <sheet name="Thiết kế dữ liệu" sheetId="8" r:id="rId8"/>
     <sheet name="Phân quyền luồng" sheetId="9" r:id="rId9"/>
+    <sheet name="Nhật ký thay đổi" sheetId="10" r:id="rId10"/>
   </sheets>
 </workbook>
 </file>
@@ -84,16 +85,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFB4C6E7"/>
+        <color rgb="FFBFBFBF"/>
       </left>
       <right style="thin">
-        <color rgb="FFB4C6E7"/>
+        <color rgb="FFBFBFBF"/>
       </right>
       <top style="thin">
-        <color rgb="FFB4C6E7"/>
+        <color rgb="FFBFBFBF"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFB4C6E7"/>
+        <color rgb="FFBFBFBF"/>
       </bottom>
       <diagonal/>
     </border>
@@ -102,23 +103,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="7">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyBorder="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyBorder="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyBorder="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyBorder="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyBorder="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -136,7 +137,7 @@
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
-    <col min="3" max="3" width="70" customWidth="1"/>
+    <col min="3" max="3" width="80" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -164,12 +165,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/10/2026</t>
+          <t xml:space="preserve">14/10/2026</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đối chiếu trực tiếp mã nguồn trên nhánh ProfessionalCode.</t>
+          <t xml:space="preserve">Đối chiếu trực tiếp mã nguồn trên nhánh main.</t>
         </is>
       </c>
     </row>
@@ -181,12 +182,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ProfessionalCode (d4a4a16)</t>
+          <t xml:space="preserve">main (c7a1964) + feat/builds-va-tim-kiem-toan-cuc</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Working tree: heroes.json đã sửa, AOV_HUB.xlsx chưa được theo dõi.</t>
+          <t xml:space="preserve">PR #57, #58 (Tướng/Trang bị nổi bật), #59 (API dữ liệu dùng chung) đã merge vào main; UI/responsive/a11y trên nhánh fix/ui-responsive-a11y (chưa merge); build + tìm kiếm toàn cục trên nhánh này.</t>
         </is>
       </c>
     </row>
@@ -227,11 +228,11 @@
         </is>
       </c>
       <c r="B6" s="2">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phủ 13/32 tướng (xem L12).</t>
+          <t xml:space="preserve">Phủ 32/32 tướng (mỗi tướng 1 build).</t>
         </is>
       </c>
     </row>
@@ -257,11 +258,11 @@
         </is>
       </c>
       <c r="B8" s="2">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">index.html + 15 trang trong src/pages.</t>
+          <t xml:space="preserve">index.html + 16 trang trong src/pages (đã thêm search.html).</t>
         </is>
       </c>
     </row>
@@ -272,11 +273,11 @@
         </is>
       </c>
       <c r="B9" s="2">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">public/css.</t>
+          <t xml:space="preserve">public/css (đã thêm hero-admin.css, search.css).</t>
         </is>
       </c>
     </row>
@@ -287,11 +288,11 @@
         </is>
       </c>
       <c r="B10" s="2">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/js (chưa kể core/adapters/services/controllers/models).</t>
+          <t xml:space="preserve">src/js top-level (chưa kể 11 file core/adapters/services/controllers/models — tổng cộng 35 file).</t>
         </is>
       </c>
     </row>
@@ -303,12 +304,12 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">16/16 file PASS + 77 E2E PASS</t>
+          <t xml:space="preserve">17/17 file PASS + 82 E2E PASS</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">mini-DOM: 16 file PASS; Playwright (trình duyệt thật): 77 PASS.</t>
+          <t xml:space="preserve">mini-DOM: 17 file PASS; Playwright (trình duyệt thật): 82 PASS.</t>
         </is>
       </c>
     </row>
@@ -320,12 +321,12 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">77/77 PASS</t>
+          <t xml:space="preserve">82/82 PASS</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">15 trang × 360/480/768/1024/1280 không tràn ngang; menu mobile hoạt động.</t>
+          <t xml:space="preserve">16 trang × 360/480/768/1024/1280 không tràn ngang; menu mobile hoạt động.</t>
         </is>
       </c>
     </row>
@@ -337,7 +338,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">16/16 trang</t>
+          <t xml:space="preserve">17/17 trang</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -353,11 +354,11 @@
         </is>
       </c>
       <c r="B14" s="2">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">STT 1-50; các mục 48, 49, 50 nay đã xong.</t>
+          <t xml:space="preserve">STT 1-50; nay thêm STT 6, 18, 29, 36 đã xong.</t>
         </is>
       </c>
     </row>
@@ -368,11 +369,11 @@
         </is>
       </c>
       <c r="B15" s="2">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">STT 6,13,18,20,29,36.</t>
+          <t xml:space="preserve">STT 13 (tách profile.js), 20 (lọc đường đi).</t>
         </is>
       </c>
     </row>
@@ -399,12 +400,12 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">L14, L15, L17, L18, L23, L24</t>
+          <t xml:space="preserve">L12, L14, L15, L17, L18, L20, L22, L23, L24</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">open redirect, băm mật khẩu, backup.rar, README, trang 404, responsive admin.</t>
+          <t xml:space="preserve">open redirect, băm mật khẩu, backup.rar, README, trang 404, responsive admin, build đủ 32 tướng, tìm kiếm toàn cục, tiêu chí nổi bật.</t>
         </is>
       </c>
     </row>
@@ -416,12 +417,12 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">L06, L12, L19, L20, L22</t>
+          <t xml:space="preserve">L06, L19</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">lane/title, build còn thiếu, tách profile.js, header search, tiêu chí nổi bật.</t>
+          <t xml:space="preserve">lane/title 32 tướng; tách code Profile thành src/js/profile.js.</t>
         </is>
       </c>
     </row>
@@ -433,12 +434,12 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">CM02, KD01, KD02, AD01-AD04, AD10</t>
+          <t xml:space="preserve">CM02, CM03, CM04, CM05, KD01, KD02, AD01-AD04, AD09, AD10</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nhật ký admin, trạng thái bài, duyệt trước, quản lý tướng CRUD.</t>
+          <t xml:space="preserve">Nhật ký admin, khung quản trị đa tab, sao lưu/khôi phục + cảnh báo dung lượng, trạng thái bài, duyệt trước, quản lý tướng CRUD, kiểm tra dữ liệu.</t>
         </is>
       </c>
     </row>
@@ -450,34 +451,660 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KD03, AD05-AD09, HD01-HD10</t>
+          <t xml:space="preserve">KD03, KD05, KD06, KD11, AD05-AD08, HD01-HD10</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Duyệt/từ chối bài, quản lý trang bị/build, hướng dẫn build.</t>
+          <t xml:space="preserve">Duyệt/từ chối bài, báo cáo, nhật ký dạng tab, quản lý trang bị/build, hướng dẫn build.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">Tab quản trị còn thiếu file</t>
+        </is>
+      </c>
+      <c r="B21" s="2">
+        <v>8</v>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">admin-shell.js khai báo 8 file tab chưa viết (admin-pending/build-review/reports/users/items/builds/log/banned.js); tab Dữ liệu đã đủ 3 file backup/storage/datacheck.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">Rủi ro chính</t>
         </is>
       </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Không backend; quyền admin chỉ ở trình duyệt</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dữ liệu ở JSON/LocalStorage/File System Access; lớp clean architecture chưa được nạp; đã có test Playwright (77 PASS) và checklist demo nhưng vẫn chỉ là demo, không phải bảo mật thật.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:C22"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="54" customWidth="1"/>
+    <col min="5" max="5" width="54" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ngày</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mã / mục</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Loại</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nội dung cập nhật</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ghi chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14/10/2026</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tổng hợp</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cập nhật mốc</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ngày review 10/10/2026 -&gt; 14/10/2026; nhánh ProfessionalCode (d4a4a16) -&gt; main (1d779ef)</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PR #57 (Responsive/Playwright) đã merge vào main.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14/10/2026</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CM03</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sửa trạng thái</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Một phần -&gt; Đã xong</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Khung quản trị đa tab admin-shell.js: menu dọc 4 nhóm, 10 tab, badge, nút 'Thoát quản lý'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14/10/2026</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CM04</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sửa trạng thái</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chưa làm -&gt; Đã xong</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sao lưu/khôi phục dữ liệu admin (Xuất/Nhập JSON) trong admin.js + #admin-backup.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14/10/2026</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CM05</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sửa trạng thái</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chưa làm -&gt; Một phần</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Có khung cảnh báo LocalStorage (#admin-notices); thiếu hàm getStorageUsage().</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14/10/2026</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KD03</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sửa trạng thái</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chưa làm -&gt; Một phần</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã có mục 'Chờ duyệt' + badge đếm bài pending; chưa có nút duyệt/từ chối.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14/10/2026</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KD11</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sửa trạng thái</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chưa làm -&gt; Một phần</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã có mục 'Nhật ký' trong khung; admin-log.js chưa viết.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14/10/2026</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KD05/KD06/KD09</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bổ sung ghi chú</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Khung đã có mục 'Báo cáo'/'Người dùng'; các file admin-reports.js/admin-users.js chưa viết.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14/10/2026</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AD05-AD09</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bổ sung ghi chú</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Khung đã có mục 'Trang bị'/'Build'/'Dữ liệu' dạng tab rỗng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14/10/2026</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">L21</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sửa trạng thái</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Một phần -&gt; Đã xong</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">16 file test mini-DOM PASS + 77 test Playwright (trình duyệt thật) PASS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14/10/2026</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">L02</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sửa ghi chú</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hero.css 12KB -&gt; ~15KB.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14/10/2026</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N08</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sửa trạng thái</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chưa làm -&gt; Đã xong</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/responsive.spec.ts; 77 test PASS trên Chromium.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14/10/2026</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N07</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sửa trạng thái</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chưa làm -&gt; Một phần</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sao lưu admin (CM04) đã bao phủ các khoá yêu thích/lịch sử.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14/10/2026</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ngoài danh sách</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Thêm dòng</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Thêm: khung quản trị đa tab, sao lưu/khôi phục admin, Playwright E2E, Vite build nhiều trang, bỏ 'Quản lý tướng'/'Đăng xuất' khỏi Header.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14/10/2026</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Việc nên làm tiếp</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dọn &amp; thêm</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bỏ 3 việc đã xong (E2E, responsive thiết bị thật, sao lưu admin); thêm P0 'viết 11 file tab admin'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14/10/2026</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">L22 / STT 6</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sửa trạng thái</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chưa làm / Một phần -&gt; Đã xong</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">home.js lọc 'featured === true' (8 tướng + 8 trang bị); ô #hero-featured; PR #58 đã merge vào main.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14/10/2026</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">L12 / STT 29</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sửa trạng thái</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chưa làm / Một phần -&gt; Đã xong</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">builds.json 13 -&gt; 32 build, phủ 32/32 tướng; test-build-page kiểm tra ID trang bị hợp lệ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14/10/2026</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">L20 / STT 18 / N01</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sửa trạng thái</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chưa làm / Một phần -&gt; Đã xong</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Thêm search.html + search-page.js + search.css; Header trỏ sang trang Tìm kiếm toàn cục; test-search-page 16 PASS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14/10/2026</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">STT 36</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sửa trạng thái</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Một phần -&gt; Đã xong</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">test-post-form kiểm tra bài mới vào collection posts của dataStore.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14/10/2026</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CM05 / AD09</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sửa trạng thái</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Một phần / Chưa làm -&gt; Đã xong</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">admin-backup/storage/datacheck.js đã có; tab Dữ liệu đủ 3 mục; 'Tab quản trị còn thiếu file' 11 -&gt; 8.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14/10/2026</t>
+        </is>
+      </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Không backend; quyền admin chỉ ở trình duyệt</t>
+          <t xml:space="preserve">Tổng hợp</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dữ liệu nằm ở JSON/LocalStorage/File System Access; lớp clean architecture chưa được nạp; đã có test Playwright trên trình duyệt thật (77 PASS) nhưng vẫn chỉ là demo, không phải bảo mật thật.</t>
+          <t xml:space="preserve">Cập nhật mốc</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">main (1d779ef) -&gt; main (c7a1964)</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PR #58 (Tướng/Trang bị nổi bật) + #59 (API dữ liệu dùng chung) đã merge; UI/responsive trên fix/ui-responsive-a11y; build + tìm kiếm trên feat/builds-va-tim-kiem-toan-cuc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14/10/2026</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Số liệu</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cập nhật</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Build 13-&gt;32; trang HTML 16-&gt;17; CSS 13-&gt;14; JS top-level 20-&gt;24; test 16-&gt;17 file + 77-&gt;82 E2E.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C21"/>
+  <autoFilter ref="A1:E22"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -491,7 +1118,7 @@
     <col min="3" max="3" width="12" customWidth="1"/>
     <col min="4" max="4" width="10" customWidth="1"/>
     <col min="5" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="66" customWidth="1"/>
+    <col min="6" max="6" width="70" customWidth="1"/>
     <col min="7" max="7" width="42" customWidth="1"/>
   </cols>
   <sheetData>
@@ -523,7 +1150,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ghi chú kiểm tra code (10/10/2026)</t>
+          <t xml:space="preserve">Ghi chú kiểm tra code (14/10/2026)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -603,7 +1230,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">header.html + layout.js; menu 7 mục, account-area.</t>
+          <t xml:space="preserve">header.html + layout.js; menu 7 mục, account-area. Đã bỏ liên kết 'Quản lý tướng' và 'Đăng xuất' khỏi header.</t>
         </is>
       </c>
     </row>
@@ -666,9 +1293,9 @@
           <t xml:space="preserve">Trang chủ: khối Tướng nổi bật render từ heroes.json</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Một phần</t>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã xong</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -678,12 +1305,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">home.js lấy 8 phần tử đầu (slice 0-8), chưa có tiêu chí nổi bật.</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Thêm trường featured hoặc tiêu chí rõ (L22).</t>
+          <t xml:space="preserve">home.js lọc trường featured === true rồi lấy 8 tướng + 8 trang bị; admin bật ở ô #hero-featured (PR #58).</t>
         </is>
       </c>
     </row>
@@ -838,7 +1460,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">logout() xoá phiên rồi về trang chủ.</t>
+          <t xml:space="preserve">logout() xoá phiên rồi về trang chủ; nút Đăng xuất nay nằm trong trang Profile, không còn ở Header.</t>
         </is>
       </c>
     </row>
@@ -986,9 +1608,9 @@
           <t xml:space="preserve">Tìm kiếm tướng theo tên (realtime)</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Một phần</t>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã xong</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -998,12 +1620,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">hero.js lọc realtime, bỏ dấu; nhận ?keyword= từ Header. Ô search Header chỉ tới Tướng.</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Mở rộng tìm kiếm toàn cục (L20/N01).</t>
+          <t xml:space="preserve">hero.js lọc realtime, bỏ dấu; nhận ?keyword=. Ô tìm kiếm Header nay trỏ sang trang Tìm kiếm toàn cục (search.html).</t>
         </is>
       </c>
     </row>
@@ -1276,9 +1893,9 @@
           <t xml:space="preserve">builds.json gắn theo hero_id</t>
         </is>
       </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Một phần</t>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã xong</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -1288,12 +1905,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">13 build, phủ 13/32 tướng.</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bổ sung build cho 19 tướng còn lại (L12).</t>
+          <t xml:space="preserve">32 build, phủ 32/32 tướng (mỗi tướng 1 build).</t>
         </is>
       </c>
     </row>
@@ -1456,9 +2068,9 @@
           <t xml:space="preserve">Form tạo bài viết và lưu</t>
         </is>
       </c>
-      <c r="C37" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Một phần</t>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã xong</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -1468,12 +2080,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tạo bài qua dataStore (aov_posts dự phòng); có duyệt trước khi đăng.</t>
-        </is>
-      </c>
-      <c r="G37" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Kiểm tra luồng liên kết với dataStore.</t>
+          <t xml:space="preserve">Tạo bài qua dataStore (collection posts); có duyệt trước; test-post-form đã kiểm tra luồng form -&gt; dataStore.</t>
         </is>
       </c>
     </row>
@@ -1897,7 +2504,7 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ghi chú cập nhật (10/10/2026)</t>
+          <t xml:space="preserve">Ghi chú cập nhật (14/10/2026)</t>
         </is>
       </c>
     </row>
@@ -2001,7 +2608,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">hero.css 12KB, đủ style hero-detail/skill/stats + 5 khối @media.</t>
+          <t xml:space="preserve">hero.css ~15KB, đủ style hero-detail/skill/stats + 5 khối @media.</t>
         </is>
       </c>
     </row>
@@ -2514,14 +3121,14 @@
           <t xml:space="preserve">Nguyễn Tuấn Anh</t>
         </is>
       </c>
-      <c r="I13" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Chưa làm</t>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã xong</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nay 13/32 tướng; 0 build thiếu mô tả.</t>
+          <t xml:space="preserve">32/32 tướng có build; mọi ID trang bị hợp lệ, 0 build thiếu mô tả.</t>
         </is>
       </c>
     </row>
@@ -2930,14 +3537,14 @@
           <t xml:space="preserve">Trần Anh Thư</t>
         </is>
       </c>
-      <c r="I21" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Chưa làm</t>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã xong</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">header.html vẫn action=heroes.html.</t>
+          <t xml:space="preserve">Header form trỏ sang search.html (tìm tướng/trang bị/build/bài viết); có test-search-page 16 PASS.</t>
         </is>
       </c>
     </row>
@@ -2964,7 +3571,7 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">tools/</t>
+          <t xml:space="preserve">tools/, tests/</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -2982,14 +3589,14 @@
           <t xml:space="preserve">Cả nhóm</t>
         </is>
       </c>
-      <c r="I22" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Một phần</t>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã xong</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đã có 15 file test (gồm auth/favorite/compare/hero-admin); chưa test trình duyệt thật.</t>
+          <t xml:space="preserve">16 file test mini-DOM PASS + 77 test Playwright (trình duyệt thật) PASS; checklist demo ở README mục 6.</t>
         </is>
       </c>
     </row>
@@ -3034,14 +3641,14 @@
           <t xml:space="preserve">Trần Anh Thư</t>
         </is>
       </c>
-      <c r="I23" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Chưa làm</t>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã xong</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">home.js vẫn dùng slice(0, 8).</t>
+          <t xml:space="preserve">home.js lọc theo featured === true (8 tướng + 8 trang bị); ô #hero-featured trong quản lý tướng.</t>
         </is>
       </c>
     </row>
@@ -3145,7 +3752,7 @@
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đã bổ sung @media 768/480 cho bảng và thanh công cụ.</t>
+          <t xml:space="preserve">Đã bổ sung 8 khối @media (768/480) cho bảng và thanh công cụ.</t>
         </is>
       </c>
     </row>
@@ -3164,7 +3771,7 @@
     <col min="3" max="3" width="46" customWidth="1"/>
     <col min="4" max="4" width="34" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="62" customWidth="1"/>
+    <col min="6" max="6" width="66" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -3195,7 +3802,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ghi chú kiểm tra (10/10/2026)</t>
+          <t xml:space="preserve">Ghi chú kiểm tra (14/10/2026)</t>
         </is>
       </c>
     </row>
@@ -3284,14 +3891,14 @@
           <t xml:space="preserve">admin.html, hero-admin.html</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Một phần</t>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã xong</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Có 2 trang admin riêng; chưa có thanh tab/badge dùng chung.</t>
+          <t xml:space="preserve">admin-shell.js: menu dọc 4 nhóm, 10 tab (posts/pending/reports/users/heroes/items/builds/log/data/settings), badge, nút 'Thoát quản lý'; hero-admin.html vào thẳng khung ở tab Tướng.</t>
         </is>
       </c>
     </row>
@@ -3316,14 +3923,14 @@
           <t xml:space="preserve">admin.html, admin.js</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Chưa làm</t>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã xong</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chưa có nút xuất/nhập JSON toàn bộ.</t>
+          <t xml:space="preserve">Nay ở tab Dữ liệu (admin-backup.js): sao lưu/khôi phục 9 khoá aov_* + nút Xuất/Nhập JSON.</t>
         </is>
       </c>
     </row>
@@ -3348,14 +3955,14 @@
           <t xml:space="preserve">storage.js, admin.html</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Chưa làm</t>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã xong</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chưa có thanh đo/cảnh báo.</t>
+          <t xml:space="preserve">admin-storage.js vẽ mục 'Dung lượng LocalStorage' dùng getStorageUsage()/formatStorageSize() (đã có trong storage.js).</t>
         </is>
       </c>
     </row>
@@ -3387,7 +3994,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Có test-hero-admin và test-datastore; chưa có test-admin-data riêng.</t>
+          <t xml:space="preserve">Có test-admin-shell, test-admin-page, test-hero-admin, test-datastore; chưa có test-admin-data/items/builds riêng.</t>
         </is>
       </c>
     </row>
@@ -3476,14 +4083,14 @@
           <t xml:space="preserve">admin.js, admin.html, feed.js</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Chưa làm</t>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Một phần</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chưa có approvePost()/rejectPost(); bảng admin mới ẩn/hiện/xoá.</t>
+          <t xml:space="preserve">Khung đã có mục 'Chờ duyệt' + badge đếm bài pending; admin-pending.js chưa viết (hiện 'Mục này đang được phát triển.'); chưa có approvePost()/rejectPost().</t>
         </is>
       </c>
     </row>
@@ -3547,7 +4154,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chưa có key aov_reports.</t>
+          <t xml:space="preserve">Chưa có key aov_reports; khung đã có mục 'Báo cáo' (chờ admin-reports.js).</t>
         </is>
       </c>
     </row>
@@ -3579,7 +4186,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">autoHideThreshold mới ở cấu hình, chưa dùng.</t>
+          <t xml:space="preserve">autoHideThreshold mới ở cấu hình, chưa dùng; badge 'Báo cáo' cần getOpenReportCount() (chưa có).</t>
         </is>
       </c>
     </row>
@@ -3675,7 +4282,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">users.json chưa có banned/warnings.</t>
+          <t xml:space="preserve">users.json chưa có banned/warnings; khung đã có mục 'Người dùng' (chờ admin-users.js).</t>
         </is>
       </c>
     </row>
@@ -3707,7 +4314,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bảng hiện badge trạng thái; chưa có bộ lọc theo trạng thái.</t>
+          <t xml:space="preserve">Bảng hiện badge trạng thái; chưa có bộ lọc theo trạng thái (chỉ có ô tìm theo tiêu đề/tác giả).</t>
         </is>
       </c>
     </row>
@@ -3732,14 +4339,14 @@
           <t xml:space="preserve">admin.js, admin.html</t>
         </is>
       </c>
-      <c r="E18" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Chưa làm</t>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Một phần</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">adminlog.js đã có; chưa có tab UI.</t>
+          <t xml:space="preserve">Khung đã có mục 'Nhật ký'; admin-log.js chưa viết (adminlog.js core đã có).</t>
         </is>
       </c>
     </row>
@@ -3798,7 +4405,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bảng, tìm theo tên, lọc vai trò, phân trang.</t>
+          <t xml:space="preserve">Nay là mục 'Tướng' trong khung quản trị: bảng, tìm theo tên, lọc vai trò, phân trang.</t>
         </is>
       </c>
     </row>
@@ -3916,7 +4523,7 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin-items.html/js</t>
+          <t xml:space="preserve">admin-items.js</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -3926,7 +4533,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chưa có.</t>
+          <t xml:space="preserve">Khung đã có mục 'Trang bị'; admin-items.js chưa viết.</t>
         </is>
       </c>
     </row>
@@ -3956,6 +4563,11 @@
           <t xml:space="preserve">Chưa làm</t>
         </is>
       </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Khung đã có mục 'Trang bị'; admin-items.js chưa viết.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -3975,12 +4587,17 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin-builds.html/js</t>
+          <t xml:space="preserve">admin-builds.js</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Chưa làm</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Khung đã có mục 'Build'; admin-builds.js chưa viết.</t>
         </is>
       </c>
     </row>
@@ -4010,6 +4627,11 @@
           <t xml:space="preserve">Chưa làm</t>
         </is>
       </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Khung đã có mục 'Build'; admin-builds.js chưa viết.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -4029,12 +4651,17 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin.js</t>
-        </is>
-      </c>
-      <c r="E28" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Chưa làm</t>
+          <t xml:space="preserve">admin-datacheck.js</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã xong</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">admin-datacheck.js (32KB) đăng ký mục 'Kiểm tra dữ liệu' trong tab Dữ liệu.</t>
         </is>
       </c>
     </row>
@@ -4098,7 +4725,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">test-hero-admin bao phủ tướng; chưa có admin-items/builds.</t>
+          <t xml:space="preserve">test-hero-admin + test-admin-shell bao phủ tướng và khung; chưa có admin-items/builds.</t>
         </is>
       </c>
     </row>
@@ -4399,7 +5026,7 @@
   <cols>
     <col min="1" max="1" width="52" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="66" customWidth="1"/>
+    <col min="3" max="3" width="70" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -4415,7 +5042,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ghi chú kiểm tra (10/10/2026)</t>
+          <t xml:space="preserve">Ghi chú kiểm tra (14/10/2026)</t>
         </is>
       </c>
     </row>
@@ -4432,7 +5059,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hiển thị 13 build, tìm theo tên tướng/build, link sang chi tiết tướng và trang bị.</t>
+          <t xml:space="preserve">Hiển thị 32 build (phủ 32/32 tướng), tìm theo tên tướng/build, link sang chi tiết tướng và trang bị.</t>
         </is>
       </c>
     </row>
@@ -4500,7 +5127,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">16 file test mini-DOM PASS; 77 test Playwright responsive PASS (trình duyệt thật).</t>
+          <t xml:space="preserve">17 file test mini-DOM PASS; 82 test Playwright responsive PASS (trình duyệt thật).</t>
         </is>
       </c>
     </row>
@@ -4534,7 +5161,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lấy từ dataStore/storage.js và feed.js; code còn inline.</t>
+          <t xml:space="preserve">Lấy từ dataStore/storage.js và feed.js; code còn inline (L19).</t>
         </is>
       </c>
     </row>
@@ -4619,7 +5246,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">File System Access API + migrate khoá LocalStorage cũ; đồng bộ nhiều tab.</t>
+          <t xml:space="preserve">API nội bộ GET/PUT /api/&lt;collection&gt; (users/posts/comments/likes/items) ghi thẳng src/data/*.json + File System Access API + migrate khoá cũ; đồng bộ nhiều tab.</t>
         </is>
       </c>
     </row>
@@ -4636,7 +5263,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">CRUD ghi thẳng heroes.json qua Vite middleware; validate + tải ảnh.</t>
+          <t xml:space="preserve">hero-admin.html nay vào thẳng khung quản trị ở tab Tướng (data-admin-tab=heroes); CRUD ghi thẳng heroes.json qua Vite middleware.</t>
         </is>
       </c>
     </row>
@@ -4694,39 +5321,175 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lớp clean architecture (core/adapters/services/controllers/models)</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Một phần</t>
+          <t xml:space="preserve">Khung quản trị đa tab (admin-shell.js + admin.html/hero-admin.html)</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã xong</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đã viết nhưng CHƯA trang nào nạp; cần tích hợp hoặc gỡ để tránh code chết.</t>
+          <t xml:space="preserve">CM03: menu dọc 4 nhóm, 10 tab, badge pending/reports, nút 'Thoát quản lý'; tab thiếu file hiện 'Mục này đang được phát triển.'.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">Sao lưu / khôi phục dữ liệu admin (Xuất/Nhập JSON)</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã xong</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CM04: admin.js exportAdminData()/handleAdminImport(); sao lưu 9 khoá aov_* (bài viết, like, bình luận, yêu thích, build, lịch sử, so sánh, cài đặt, nhật ký).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Test E2E Playwright (tests/responsive.spec.ts + playwright.config.ts)</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã xong</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N08: 82 test PASS trên Chromium (trình duyệt thật).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đóng gói Vite nhiều trang (vite.config.js)</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã xong</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">17 trang; chép src/js + src/data vào dist; kiểm tra bằng npm run preview (tất cả URL trả 200).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rời 'Quản lý tướng' / 'Đăng xuất' khỏi Header</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã xong</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đăng xuất nay nằm trong trang Profile; header còn menu 7 mục + tìm kiếm + account-area.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lớp clean architecture (core/adapters/services/controllers/models)</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Một phần</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã viết nhưng CHƯA trang nào nạp; cần tích hợp hoặc gỡ để tránh code chết.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">config.js, heroData.js, search.js dùng chung</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Đã xong</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã xong</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">BASE_PATH/DATA_PATH; lớp dữ liệu tướng; chuẩn hoá từ khoá bỏ dấu.</t>
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Trang Tìm kiếm toàn cục (search.html + search-page.js + search.css)</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã xong</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ô tìm kiếm Header trỏ sang đây; gom 4 nhóm Tướng/Trang bị/Build/Bài viết; bỏ dấu; đồng bộ ?keyword= (L20/N01).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mục 'Dữ liệu' trong khung quản trị (admin-backup/storage/datacheck.js)</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã xong</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đủ 3 mục con: Sao lưu &amp; khôi phục, Dung lượng LocalStorage (getStorageUsage), Kiểm tra dữ liệu (AD09/CM05).</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chuẩn hoá design token + breakpoint + trợ năng (nhánh fix/ui-responsive-a11y)</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã xong (chưa merge)</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đưa hex/rgba về var(--color-*); breakpoint 1200/1024/900/768/480; menu mobile &lt;button&gt; aria-expanded; aria-current; role=status; ảnh có width/height.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C19"/>
+  <autoFilter ref="A1:C27"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -4812,9 +5575,9 @@
           <t xml:space="preserve">L20</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Chưa làm</t>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã xong</t>
         </is>
       </c>
     </row>
@@ -5031,12 +5794,12 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">storage.js</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Chưa làm</t>
+          <t xml:space="preserve">storage.js, CM04</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Một phần</t>
         </is>
       </c>
     </row>
@@ -5071,9 +5834,9 @@
           <t xml:space="preserve">L21</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Chưa làm</t>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã xong</t>
         </is>
       </c>
     </row>
@@ -5267,49 +6030,49 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tab Chờ duyệt + approvePost()/rejectPost() (duyệt/từ chối kèm lý do)</t>
+          <t xml:space="preserve">Viết 8 file tab admin còn thiếu để bỏ placeholder 'Mục này đang được phát triển.'</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KD03</t>
+          <t xml:space="preserve">CM03, KD03, KD11, AD05-AD08</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/js/admin.js, admin.html, feed.js</t>
+          <t xml:space="preserve">src/js/admin-pending/build-review/reports/users/items/builds/log/banned.js</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">8 giờ</t>
+          <t xml:space="preserve">16-24 giờ</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">P1</t>
+          <t xml:space="preserve">P0</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Thêm lane + title cho 32 tướng + select lọc đường đi</t>
+          <t xml:space="preserve">Tab Chờ duyệt + approvePost()/rejectPost() (duyệt/từ chối kèm lý do) — nối vào mục 'Chờ duyệt' đã có</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">L06</t>
+          <t xml:space="preserve">KD03</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/data/heroes.json, hero.js, hero-admin.js</t>
+          <t xml:space="preserve">src/js/admin-pending.js, admin.js, feed.js</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 giờ</t>
+          <t xml:space="preserve">8 giờ</t>
         </is>
       </c>
     </row>
@@ -5321,17 +6084,17 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bổ sung build cho 19 tướng còn lại</t>
+          <t xml:space="preserve">Thêm lane + title cho 32 tướng + select lọc đường đi</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">L12</t>
+          <t xml:space="preserve">L06</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/data/builds.json</t>
+          <t xml:space="preserve">src/data/heroes.json, hero.js, hero-admin.js</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -5348,22 +6111,22 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tìm kiếm toàn cục ở Header (tướng/trang bị/build/bài viết)</t>
+          <t xml:space="preserve">Tách src/js/profile.js khỏi profile.html</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">L20, N01</t>
+          <t xml:space="preserve">L19</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">header.html, search.js</t>
+          <t xml:space="preserve">src/js/profile.js</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">6 giờ</t>
+          <t xml:space="preserve">2 giờ</t>
         </is>
       </c>
     </row>
@@ -5375,130 +6138,130 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tách src/js/profile.js khỏi profile.html</t>
+          <t xml:space="preserve">Báo cáo vi phạm (aov_reports) + tab xử lý cho admin</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">L19</t>
+          <t xml:space="preserve">KD05, KD06</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/js/profile.js</t>
+          <t xml:space="preserve">feed.js, admin-reports.js</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2 giờ</t>
+          <t xml:space="preserve">12 giờ</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">P1</t>
+          <t xml:space="preserve">P2</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tiêu chí Tướng/Trang bị nổi bật cho trang chủ</t>
+          <t xml:space="preserve">Quản lý Trang bị (form thêm/sửa/xoá an toàn)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">L22</t>
+          <t xml:space="preserve">AD05, AD06</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/js/home.js</t>
+          <t xml:space="preserve">admin-items.js</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2 giờ</t>
+          <t xml:space="preserve">16 giờ</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">P1</t>
+          <t xml:space="preserve">P2</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Báo cáo vi phạm (aov_reports) + tab xử lý cho admin</t>
+          <t xml:space="preserve">Quản lý Build + danh sách tướng thiếu build</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KD05, KD06</t>
+          <t xml:space="preserve">AD07, AD08</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">feed.js, admin.js</t>
+          <t xml:space="preserve">admin-builds.js</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">12 giờ</t>
+          <t xml:space="preserve">11 giờ</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">P1</t>
+          <t xml:space="preserve">P2</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Test E2E trên trình duyệt thật + checklist demo</t>
+          <t xml:space="preserve">Trang chi tiết hướng dẫn build + mở rộng builds.json</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">L21, N08</t>
+          <t xml:space="preserve">HD01, HD02</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">tools/</t>
+          <t xml:space="preserve">build-detail.html/js, builds.json</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">6 giờ</t>
+          <t xml:space="preserve">13 giờ</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">P1</t>
+          <t xml:space="preserve">P2</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kiểm tra responsive trên thiết bị thật (điện thoại/tablet)</t>
+          <t xml:space="preserve">Áp dụng bộ lọc từ khoá cấm vào nội dung</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">48, 49</t>
+          <t xml:space="preserve">KD07</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">public/css/*</t>
+          <t xml:space="preserve">feed.js, search.js</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 giờ</t>
+          <t xml:space="preserve">5 giờ</t>
         </is>
       </c>
     </row>
@@ -5510,22 +6273,22 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quản lý Trang bị (form thêm/sửa/xoá an toàn)</t>
+          <t xml:space="preserve">Kiểm duyệt bình luận (trường hidden + UI admin)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">AD05, AD06</t>
+          <t xml:space="preserve">KD08</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin-items.html/js</t>
+          <t xml:space="preserve">feed.js, admin.js</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">16 giờ</t>
+          <t xml:space="preserve">5 giờ</t>
         </is>
       </c>
     </row>
@@ -5537,22 +6300,22 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quản lý Build + danh sách tướng thiếu build</t>
+          <t xml:space="preserve">Quản lý người dùng: khoá / cảnh cáo</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">AD07, AD08</t>
+          <t xml:space="preserve">KD09</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin-builds.html/js</t>
+          <t xml:space="preserve">auth.js, admin-users.js</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">11 giờ</t>
+          <t xml:space="preserve">6 giờ</t>
         </is>
       </c>
     </row>
@@ -5564,351 +6327,189 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trang chi tiết hướng dẫn build + mở rộng builds.json</t>
+          <t xml:space="preserve">Tab Nhật ký admin (dùng adminlog.js đã có)</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HD01, HD02</t>
+          <t xml:space="preserve">CM02, KD11</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">build-detail.html/js, builds.json</t>
+          <t xml:space="preserve">admin-log.js</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">13 giờ</t>
+          <t xml:space="preserve">3 giờ</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">P2</t>
+          <t xml:space="preserve">P3</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Áp dụng bộ lọc từ khoá cấm vào nội dung</t>
+          <t xml:space="preserve">Trình dựng build + chia sẻ link + bình chọn Hữu ích</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KD07</t>
+          <t xml:space="preserve">N02, N05, HD07, HD09</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">feed.js, search.js</t>
+          <t xml:space="preserve">build.js, build-detail.js</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">5 giờ</t>
+          <t xml:space="preserve">12 giờ</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">P2</t>
+          <t xml:space="preserve">P3</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kiểm duyệt bình luận (trường hidden + UI admin)</t>
+          <t xml:space="preserve">Dark/Light mode</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KD08</t>
+          <t xml:space="preserve">N03</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">feed.js, admin.js</t>
+          <t xml:space="preserve">variables.css, layout.js</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">5 giờ</t>
+          <t xml:space="preserve">3 giờ</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">P2</t>
+          <t xml:space="preserve">P3</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quản lý người dùng: khoá / cảnh cáo</t>
+          <t xml:space="preserve">So sánh trang bị</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KD09</t>
+          <t xml:space="preserve">N04</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">auth.js, admin.js</t>
+          <t xml:space="preserve">compare.js</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">6 giờ</t>
+          <t xml:space="preserve">4 giờ</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">P2</t>
+          <t xml:space="preserve">P3</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tab Nhật ký admin (dùng adminlog.js đã có)</t>
+          <t xml:space="preserve">Biểu đồ radar chỉ số tướng</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">CM02, KD11</t>
+          <t xml:space="preserve">N06</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin.html, admin.js</t>
+          <t xml:space="preserve">hero-detail, compare</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 giờ</t>
+          <t xml:space="preserve">6 giờ</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">P2</t>
+          <t xml:space="preserve">P3</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sao lưu / khôi phục dữ liệu admin</t>
+          <t xml:space="preserve">Xuất / nhập dữ liệu người dùng</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">CM04</t>
+          <t xml:space="preserve">N07</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin.html, admin.js</t>
+          <t xml:space="preserve">storage.js</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 giờ</t>
+          <t xml:space="preserve">3 giờ</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">P2</t>
+          <t xml:space="preserve">P3</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cảnh báo dung lượng LocalStorage</t>
+          <t xml:space="preserve">PWA + đa ngôn ngữ</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">CM05</t>
+          <t xml:space="preserve">N10, N11</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">storage.js, admin.html</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2 giờ</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P3</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Trình dựng build + chia sẻ link + bình chọn Hữu ích</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">N02, N05, HD07, HD09</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">build.js, build-detail.js</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">12 giờ</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P3</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Dark/Light mode</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">N03</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">variables.css, layout.js</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3 giờ</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P3</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">So sánh trang bị</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">N04</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">compare.js</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4 giờ</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P3</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Biểu đồ radar chỉ số tướng</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">N06</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">hero-detail, compare</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6 giờ</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P3</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Xuất / nhập dữ liệu người dùng</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">N07</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">storage.js</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3 giờ</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P3</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PWA + đa ngôn ngữ</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">N10, N11</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
           <t xml:space="preserve">16 giờ</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E26"/>
+  <autoFilter ref="A1:E20"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -5921,7 +6522,7 @@
     <col min="2" max="2" width="30" customWidth="1"/>
     <col min="3" max="3" width="46" customWidth="1"/>
     <col min="4" max="4" width="18" customWidth="1"/>
-    <col min="5" max="5" width="40" customWidth="1"/>
+    <col min="5" max="5" width="44" customWidth="1"/>
     <col min="6" max="6" width="30" customWidth="1"/>
   </cols>
   <sheetData>
@@ -6145,56 +6746,56 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đã triển khai (chưa có tab UI)</t>
+          <t xml:space="preserve">Đã triển khai (chưa có tab UI — KD11)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tướng</t>
+          <t xml:space="preserve">Bản sao lưu admin</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">heroes.json (ghi qua API /api/heroes)</t>
+          <t xml:space="preserve">File JSON tải về (aov-hub-backup-*.json)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">id, name, alias, image, role, difficulty, stats, skills, recommendedBuild</t>
+          <t xml:space="preserve">meta{app, exportedAt, version} + data{aov_posts, aov_mod_settings, aov_likes, aov_comments, aov_favorites, aov_builds, aov_hero_history, aov_hero_compare, aov_admin_log}</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">hỗn hợp</t>
+          <t xml:space="preserve">object</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">32 tướng; admin CRUD ghi thẳng file JSON</t>
+          <t xml:space="preserve">Xuất/nhập toàn bộ qua admin.js; khôi phục ghi đè localStorage rồi tải lại trang</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đã triển khai; thiếu lane, title (L06)</t>
+          <t xml:space="preserve">Đã triển khai (CM04)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trang bị</t>
+          <t xml:space="preserve">Tướng</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">items.json</t>
+          <t xml:space="preserve">heroes.json (ghi qua API /api/heroes)</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">id, name, alias, image, type, price, stats, passive, description, related</t>
+          <t xml:space="preserve">id, name, alias, image, role, difficulty, stats, skills, recommendedBuild</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -6204,29 +6805,29 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40 trang bị; ID theo nhóm 1xx-6xx</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Đã triển khai</t>
+          <t xml:space="preserve">32 tướng; admin CRUD ghi thẳng file JSON</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã triển khai; thiếu lane, title (L06)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Build</t>
+          <t xml:space="preserve">Trang bị</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">builds.json</t>
+          <t xml:space="preserve">items.json</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">id, heroId, name, items, description</t>
+          <t xml:space="preserve">id, name, alias, image, type, price, stats, passive, description, related</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -6236,71 +6837,71 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">13 build; chưa mở rộng thành hướng dẫn</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Đã triển khai; chờ mở rộng (HD01)</t>
+          <t xml:space="preserve">40 trang bị; ID theo nhóm 1xx-6xx</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã triển khai</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bản nháp dataStore</t>
+          <t xml:space="preserve">Build</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">aov_draft_* + IndexedDB aov-datastore</t>
+          <t xml:space="preserve">builds.json</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">handle thư mục src/data</t>
+          <t xml:space="preserve">id, heroId, name, items, description</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">hỗn hợp</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lưu nháp khi chưa liên kết thư mục; đồng bộ nhiều tab qua BroadcastChannel aov-data</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Đã triển khai</t>
+          <t xml:space="preserve">32 build (phủ 32/32 tướng); chưa mở rộng thành hướng dẫn</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã triển khai; chờ mở rộng (HD01)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yêu thích</t>
+          <t xml:space="preserve">Bản nháp dataStore</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">aov_favorites (LocalStorage)</t>
+          <t xml:space="preserve">aov_draft_* + IndexedDB aov-datastore</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">{ hero: [id], item: [id] }</t>
+          <t xml:space="preserve">handle thư mục src/data</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">object</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Không đổi tên key; chưa có nhóm build</t>
+          <t xml:space="preserve">Lưu nháp khi chưa liên kết thư mục; đồng bộ nhiều tab qua BroadcastChannel aov-data</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
@@ -6312,165 +6913,197 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Báo cáo</t>
+          <t xml:space="preserve">Yêu thích</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">aov_reports</t>
+          <t xml:space="preserve">aov_favorites (LocalStorage)</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">id, targetType, targetId, reporter, reason, note, createdAt, status, handledBy</t>
+          <t xml:space="preserve">{ hero: [id], item: [id] }</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">hỗn hợp</t>
+          <t xml:space="preserve">object</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Báo cáo bài/bình luận vi phạm</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CHƯA triển khai (kế hoạch KD05/KD06)</t>
+          <t xml:space="preserve">Không đổi tên key; chưa có nhóm build</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã triển khai</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bình chọn build</t>
+          <t xml:space="preserve">Báo cáo</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">aov_build_votes</t>
+          <t xml:space="preserve">aov_reports</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">{ buildId: [username] }</t>
+          <t xml:space="preserve">id, targetType, targetId, reporter, reason, note, createdAt, status, handledBy</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">object</t>
+          <t xml:space="preserve">hỗn hợp</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mỗi người một lượt/build</t>
+          <t xml:space="preserve">Báo cáo bài/bình luận vi phạm</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">CHƯA triển khai (kế hoạch HD07)</t>
+          <t xml:space="preserve">CHƯA triển khai (kế hoạch KD05/KD06)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tướng/Trang bị/Build mở rộng</t>
+          <t xml:space="preserve">Bình chọn build</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">aov_heroes_ext / aov_items_ext / aov_builds_ext</t>
+          <t xml:space="preserve">aov_build_votes</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">added/edited/deleted</t>
+          <t xml:space="preserve">{ buildId: [username] }</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">hỗn hợp</t>
+          <t xml:space="preserve">object</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lớp gộp overrides lên JSON gốc</t>
+          <t xml:space="preserve">Mỗi người một lượt/build</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KHÔNG dùng: thay bằng dataStore + API /api/heroes</t>
+          <t xml:space="preserve">CHƯA triển khai (kế hoạch HD07)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Người dùng (khóa/cảnh cáo)</t>
+          <t xml:space="preserve">Tướng/Trang bị/Build mở rộng</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">aov_users / users.json</t>
+          <t xml:space="preserve">aov_heroes_ext / aov_items_ext / aov_builds_ext</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">banned, bannedReason, warnings</t>
+          <t xml:space="preserve">added/edited/deleted</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">boolean/chuỗi/số</t>
+          <t xml:space="preserve">hỗn hợp</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Khoá tài khoản và số lần cảnh cáo</t>
+          <t xml:space="preserve">Lớp gộp overrides lên JSON gốc</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">CHƯA triển khai (kế hoạch KD09)</t>
+          <t xml:space="preserve">KHÔNG dùng: thay bằng dataStore + API /api/heroes</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">Người dùng (khóa/cảnh cáo)</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">aov_users / users.json</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">banned, bannedReason, warnings</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">boolean/chuỗi/số</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Khoá tài khoản và số lần cảnh cáo</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CHƯA triển khai (kế hoạch KD09)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">Giới hạn kỹ thuật</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Không backend: mọi dữ liệu ở JSON/LocalStorage/File System Access; quyền admin chỉ ở trình duyệt. Muốn dùng thật cần server + CSDL + xác thực.</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Nên ghi rõ trong báo cáo và demo</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F17"/>
+  <autoFilter ref="A1:F18"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -6485,7 +7118,7 @@
     <col min="4" max="4" width="14" customWidth="1"/>
     <col min="5" max="5" width="8" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="44" customWidth="1"/>
+    <col min="7" max="7" width="46" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -6775,14 +7408,14 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KD03: chưa có approvePost()/rejectPost().</t>
+          <t xml:space="preserve">KD03: mục 'Chờ duyệt' đã có trong khung nhưng chưa có approvePost()/rejectPost().</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Báo cáo bài / bình luận</t>
+          <t xml:space="preserve">Sao lưu / Khôi phục dữ liệu</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -6792,34 +7425,34 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">Không</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Không</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">Có</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Không</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Có</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Chưa làm</t>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã có</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KD05: chưa có aov_reports.</t>
+          <t xml:space="preserve">Xuất/Nhập JSON ở #admin-backup (admin.js).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Xem và xử lý báo cáo</t>
+          <t xml:space="preserve">Báo cáo bài / bình luận</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -6829,14 +7462,14 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">Có</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">Không</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Không</t>
-        </is>
-      </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Có</t>
@@ -6849,14 +7482,14 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KD06.</t>
+          <t xml:space="preserve">KD05: chưa có aov_reports (khung đã có mục 'Báo cáo').</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quản lý từ cấm, ngưỡng tự ẩn</t>
+          <t xml:space="preserve">Xem và xử lý báo cáo</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -6886,14 +7519,14 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KD07: mới lưu cấu hình, chưa áp dụng.</t>
+          <t xml:space="preserve">KD06: chờ admin-reports.js + getOpenReportCount().</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Khoá / mở khoá tài khoản</t>
+          <t xml:space="preserve">Quản lý từ cấm, ngưỡng tự ẩn</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -6923,14 +7556,14 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KD09: không khoá chính mình hoặc admin khác.</t>
+          <t xml:space="preserve">KD07: mới lưu cấu hình, chưa áp dụng.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Thêm / sửa / xoá Tướng</t>
+          <t xml:space="preserve">Khoá / mở khoá tài khoản</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -6953,21 +7586,21 @@
           <t xml:space="preserve">Có</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Đã có</t>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chưa làm</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">hero-admin.js + /api/heroes; canManageHeroes().</t>
+          <t xml:space="preserve">KD09: chờ admin-users.js; không khoá chính mình hoặc admin khác.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Thêm / sửa / xoá Trang bị</t>
+          <t xml:space="preserve">Thêm / sửa / xoá Tướng</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -6990,21 +7623,21 @@
           <t xml:space="preserve">Có</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Chưa làm</t>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã có</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">AD05/AD06.</t>
+          <t xml:space="preserve">tab Tướng (hero-admin.js) + /api/heroes; canManageHeroes().</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Thêm / sửa / xoá Build</t>
+          <t xml:space="preserve">Thêm / sửa / xoá Trang bị</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -7034,56 +7667,56 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">AD07.</t>
+          <t xml:space="preserve">AD05/AD06: mục 'Trang bị' đã có trong khung; admin-items.js chưa viết.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Xem build đã duyệt và hướng dẫn</t>
+          <t xml:space="preserve">Thêm / sửa / xoá Build</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">Không</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Không</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Không</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">Có</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Có</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Có</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Có</t>
-        </is>
-      </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Đã có</t>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chưa làm</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">builds.html.</t>
+          <t xml:space="preserve">AD07: mục 'Build' đã có trong khung; admin-builds.js chưa viết.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gửi hướng dẫn build</t>
+          <t xml:space="preserve">Xem build đã duyệt và hướng dẫn</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Không</t>
+          <t xml:space="preserve">Có</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -7101,21 +7734,21 @@
           <t xml:space="preserve">Có</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Chưa làm</t>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã có</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HD06.</t>
+          <t xml:space="preserve">builds.html.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bình chọn Hữu ích cho build</t>
+          <t xml:space="preserve">Gửi hướng dẫn build</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -7145,49 +7778,86 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HD07: mỗi người 1 lượt/build.</t>
+          <t xml:space="preserve">HD06.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">Bình chọn Hữu ích cho build</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Không</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Có</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Có</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Có</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chưa làm</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HD07: mỗi người 1 lượt/build.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">Xem nhật ký admin</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Không</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Không</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Không</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Có</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr">
+      <c r="F20" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Một phần</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">adminlog.js đã có; chưa có tab UI (KD11).</t>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">adminlog.js đã có + mục 'Nhật ký' trong khung; chưa có tab UI (KD11).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G19"/>
+  <autoFilter ref="A1:G20"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(excel): cap nhat AOV_HUB.xlsx (STT13, L05, L19 da xong)
- STT13/L19: tach profile.js -> Da xong
- L05: sap xep tuong A-Z/Z-A -> Da xong
- JS top-level 24 -> 25; 'lam mot phan' 2 -> 1; 'loi con ton' -> L06
- bo 1 viec da xong khoi 'Viec nen lam tiep'; them dong nhat ky thay doi
</commit_message>
<xml_diff>
--- a/AOV_HUB.xlsx
+++ b/AOV_HUB.xlsx
@@ -165,12 +165,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">14/10/2026</t>
+          <t xml:space="preserve">15/10/2026</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đối chiếu trực tiếp mã nguồn trên nhánh main.</t>
+          <t xml:space="preserve">Đối chiếu trực tiếp mã nguồn trên nhánh fix/ui-review-minor (HEAD aec1ed5).</t>
         </is>
       </c>
     </row>
@@ -182,12 +182,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">main (c7a1964) + feat/builds-va-tim-kiem-toan-cuc</t>
+          <t xml:space="preserve">fix/ui-review-minor (aec1ed5)</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PR #57, #58 (Tướng/Trang bị nổi bật), #59 (API dữ liệu dùng chung) đã merge vào main; UI/responsive/a11y trên nhánh fix/ui-responsive-a11y (chưa merge); build + tìm kiếm toàn cục trên nhánh này.</t>
+          <t xml:space="preserve">PR #60 (UI/responsive/a11y - nhánh fix/ui-responsive-a11y) và #61 (build đủ 32 tướng + Tìm kiếm toàn cục) đã merge vào main; trên nhánh này còn 3 commit refactor sau lần cập nhật Excel trước (ae278f2, 01585e4, aec1ed5).</t>
         </is>
       </c>
     </row>
@@ -243,11 +243,11 @@
         </is>
       </c>
       <c r="B7" s="2">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kèm category và heroId.</t>
+          <t xml:space="preserve">10 bài seed + 1 bài test phát sinh khi chạy app (id 1792001024923, chưa commit); likes.json có khoá tương ứng.</t>
         </is>
       </c>
     </row>
@@ -288,11 +288,11 @@
         </is>
       </c>
       <c r="B10" s="2">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/js top-level (chưa kể 11 file core/adapters/services/controllers/models — tổng cộng 35 file).</t>
+          <t xml:space="preserve">src/js top-level (chưa kể 11 file core/adapters/services/controllers/models — tổng cộng 36 file); thêm profile.js (tách từ profile.html).</t>
         </is>
       </c>
     </row>
@@ -354,11 +354,11 @@
         </is>
       </c>
       <c r="B14" s="2">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">STT 1-50; nay thêm STT 6, 18, 29, 36 đã xong.</t>
+          <t xml:space="preserve">STT 1-50; nay thêm STT 6, 13, 18, 29, 36 đã xong.</t>
         </is>
       </c>
     </row>
@@ -369,11 +369,11 @@
         </is>
       </c>
       <c r="B15" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">STT 13 (tách profile.js), 20 (lọc đường đi).</t>
+          <t xml:space="preserve">STT 20 (lọc đường đi — chờ thêm lane).</t>
         </is>
       </c>
     </row>
@@ -400,12 +400,12 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">L12, L14, L15, L17, L18, L20, L22, L23, L24</t>
+          <t xml:space="preserve">L05, L12, L14, L15, L17, L18, L19, L20, L22, L23, L24</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">open redirect, băm mật khẩu, backup.rar, README, trang 404, responsive admin, build đủ 32 tướng, tìm kiếm toàn cục, tiêu chí nổi bật.</t>
+          <t xml:space="preserve">sắp xếp tướng A-Z/Z-A (bỏ giá), open redirect, băm mật khẩu, backup.rar, README, tách profile.js, trang 404, responsive admin, build đủ 32 tướng, tìm kiếm toàn cục, tiêu chí nổi bật.</t>
         </is>
       </c>
     </row>
@@ -417,12 +417,12 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">L06, L19</t>
+          <t xml:space="preserve">L06</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">lane/title 32 tướng; tách code Profile thành src/js/profile.js.</t>
+          <t xml:space="preserve">lane/title 32 tướng.</t>
         </is>
       </c>
     </row>
@@ -488,7 +488,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dữ liệu ở JSON/LocalStorage/File System Access; lớp clean architecture chưa được nạp; đã có test Playwright (77 PASS) và checklist demo nhưng vẫn chỉ là demo, không phải bảo mật thật.</t>
+          <t xml:space="preserve">Dữ liệu ở JSON/LocalStorage/File System Access; lớp clean architecture chưa được nạp; đã có test Playwright (82 PASS) và checklist demo nhưng vẫn chỉ là demo, không phải bảo mật thật.</t>
         </is>
       </c>
     </row>
@@ -1103,8 +1103,278 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tổng hợp</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cập nhật mốc</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">main (c7a1964) -&gt; fix/ui-review-minor (aec1ed5)</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PR #60 + #61 đã merge; trên nhánh còn 3 commit refactor ae278f2, 01585e4, aec1ed5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PR #60 / L21 / N08</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sửa trạng thái</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã xong (chưa merge) -&gt; Đã xong</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nhánh fix/ui-responsive-a11y merge: design token var(--color-*), breakpoint 1200/1024/900/768/480, menu mobile aria-expanded, aria-current, role=status.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PR #61 / L12, L20, STT18/29/36, N01</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sửa trạng thái</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Build 32/32 tướng + trang Tìm kiếm toàn cục đã merge vào main.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ae278f2</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Refactor UI</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chia sẻ .page-head/.page-head__count từ build.css sang common.css; thêm aria-live cho #search-count và #search-results.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">01585e4</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Refactor JS</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">storage.js gỡ addCompare()/clearCompare() trùng; layout.js thêm kiểm tra response.ok; search-page.js đổi tên hàm và đơn giản hoá lọc bài viết.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">aec1ed5</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Refactor admin</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gỡ UI 'Sao lưu/Khôi phục' trùng ở tab Bài viết (admin.html + admin.js, -182 dòng) vì đã có trong tab Dữ liệu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Số liệu</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cập nhật</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">posts.json 10 -&gt; 11 bài (1 bài test khi chạy app); bỏ 'chưa merge' ở dòng chuẩn hoá design token; đồng bộ E2E 82 PASS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">STT 13 / L19</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sửa trạng thái</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Một phần / Chưa làm -&gt; Đã xong</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tách code Profile khỏi profile.html sang src/js/profile.js (renderProfileHeader/Stats/Posts + logout); profile.html chỉ còn nạp script; feed.js vẫn gọi renderProfilePosts(). test-admin-page 72 PASS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">L05 / STT 21</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sửa trạng thái</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Một phần / Đã xong -&gt; Đã xong</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sắp xếp tướng có select #hero-sort-filter (Mặc định/A-Z/Z-A) ghi lên URL; gỡ hàm syncHeroFilterUrl trùng trong hero.js; không còn tiêu chí giá. test-heroes-page 25 PASS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tổng hợp</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cập nhật số liệu</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Số file JS top-level 24 -&gt; 25 (thêm profile.js, tổng 36 file); 'Công việc chính làm một phần' 2 -&gt; 1 (chỉ còn STT 20); 'Lỗi còn tồn' L06, L19 -&gt; L06; bỏ 1 việc ở 'Việc nên làm tiếp'.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E22"/>
+  <autoFilter ref="A1:E32"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1473,9 +1743,9 @@
           <t xml:space="preserve">Trang Profile: thông tin + bài đã đăng</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Một phần</t>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã xong</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1485,12 +1755,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Có thông tin, thống kê, bài đã đăng nhưng code còn inline trong profile.html.</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tách thành src/js/profile.js (L19).</t>
+          <t xml:space="preserve">Đã tách code khỏi profile.html sang src/js/profile.js (currentUsername + renderProfileHeader/Stats/Posts + logout); feed.js gọi lại renderProfilePosts() như cũ.</t>
         </is>
       </c>
     </row>
@@ -2430,7 +2695,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">16 file test mini-DOM PASS; 77 test Playwright PASS; build 16 trang; checklist demo ở README (mục 6).</t>
+          <t xml:space="preserve">17 file test mini-DOM PASS; 82 test Playwright PASS; build 17 trang; checklist demo ở README (mục 6).</t>
         </is>
       </c>
     </row>
@@ -2757,14 +3022,14 @@
           <t xml:space="preserve">Trần Gia Bảo</t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Một phần</t>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã xong</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đã có A-Z/Z-A; bỏ sắp theo giá (tướng không có giá).</t>
+          <t xml:space="preserve">Select #hero-sort-filter (Mặc định/A-Z/Z-A) ghi lên URL; đã gỡ hàm syncHeroFilterUrl trùng; không còn tiêu chí giá; test-heroes-page 25 PASS.</t>
         </is>
       </c>
     </row>
@@ -3485,14 +3750,14 @@
           <t xml:space="preserve">Trần Anh Thư</t>
         </is>
       </c>
-      <c r="I20" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Chưa làm</t>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã xong</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">profile.html vẫn nạp script inline; chưa có src/js/profile.js.</t>
+          <t xml:space="preserve">Đã tạo src/js/profile.js; profile.html chỉ còn nạp &lt;script src="/src/js/profile.js"&gt;; test-admin-page 72 PASS.</t>
         </is>
       </c>
     </row>
@@ -5161,7 +5426,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lấy từ dataStore/storage.js và feed.js; code còn inline (L19).</t>
+          <t xml:space="preserve">Lấy từ dataStore/storage.js và feed.js; code đã tách sang src/js/profile.js (L19).</t>
         </is>
       </c>
     </row>
@@ -5477,14 +5742,14 @@
           <t xml:space="preserve">Chuẩn hoá design token + breakpoint + trợ năng (nhánh fix/ui-responsive-a11y)</t>
         </is>
       </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Đã xong (chưa merge)</t>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã xong</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đưa hex/rgba về var(--color-*); breakpoint 1200/1024/900/768/480; menu mobile &lt;button&gt; aria-expanded; aria-current; role=status; ảnh có width/height.</t>
+          <t xml:space="preserve">Đưa hex/rgba về var(--color-*); breakpoint 1200/1024/900/768/480; menu mobile &lt;button&gt; aria-expanded; aria-current; role=status; ảnh có width/height. Đã merge qua PR #60.</t>
         </is>
       </c>
     </row>
@@ -6111,49 +6376,49 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tách src/js/profile.js khỏi profile.html</t>
+          <t xml:space="preserve">Báo cáo vi phạm (aov_reports) + tab xử lý cho admin</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">L19</t>
+          <t xml:space="preserve">KD05, KD06</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/js/profile.js</t>
+          <t xml:space="preserve">feed.js, admin-reports.js</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2 giờ</t>
+          <t xml:space="preserve">12 giờ</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">P1</t>
+          <t xml:space="preserve">P2</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Báo cáo vi phạm (aov_reports) + tab xử lý cho admin</t>
+          <t xml:space="preserve">Quản lý Trang bị (form thêm/sửa/xoá an toàn)</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KD05, KD06</t>
+          <t xml:space="preserve">AD05, AD06</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">feed.js, admin-reports.js</t>
+          <t xml:space="preserve">admin-items.js</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">12 giờ</t>
+          <t xml:space="preserve">16 giờ</t>
         </is>
       </c>
     </row>
@@ -6165,22 +6430,22 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quản lý Trang bị (form thêm/sửa/xoá an toàn)</t>
+          <t xml:space="preserve">Quản lý Build + danh sách tướng thiếu build</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">AD05, AD06</t>
+          <t xml:space="preserve">AD07, AD08</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin-items.js</t>
+          <t xml:space="preserve">admin-builds.js</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">16 giờ</t>
+          <t xml:space="preserve">11 giờ</t>
         </is>
       </c>
     </row>
@@ -6192,22 +6457,22 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quản lý Build + danh sách tướng thiếu build</t>
+          <t xml:space="preserve">Trang chi tiết hướng dẫn build + mở rộng builds.json</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">AD07, AD08</t>
+          <t xml:space="preserve">HD01, HD02</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin-builds.js</t>
+          <t xml:space="preserve">build-detail.html/js, builds.json</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">11 giờ</t>
+          <t xml:space="preserve">13 giờ</t>
         </is>
       </c>
     </row>
@@ -6219,22 +6484,22 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trang chi tiết hướng dẫn build + mở rộng builds.json</t>
+          <t xml:space="preserve">Áp dụng bộ lọc từ khoá cấm vào nội dung</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HD01, HD02</t>
+          <t xml:space="preserve">KD07</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">build-detail.html/js, builds.json</t>
+          <t xml:space="preserve">feed.js, search.js</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">13 giờ</t>
+          <t xml:space="preserve">5 giờ</t>
         </is>
       </c>
     </row>
@@ -6246,17 +6511,17 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Áp dụng bộ lọc từ khoá cấm vào nội dung</t>
+          <t xml:space="preserve">Kiểm duyệt bình luận (trường hidden + UI admin)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KD07</t>
+          <t xml:space="preserve">KD08</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">feed.js, search.js</t>
+          <t xml:space="preserve">feed.js, admin.js</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -6273,22 +6538,22 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kiểm duyệt bình luận (trường hidden + UI admin)</t>
+          <t xml:space="preserve">Quản lý người dùng: khoá / cảnh cáo</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KD08</t>
+          <t xml:space="preserve">KD09</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">feed.js, admin.js</t>
+          <t xml:space="preserve">auth.js, admin-users.js</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">5 giờ</t>
+          <t xml:space="preserve">6 giờ</t>
         </is>
       </c>
     </row>
@@ -6300,49 +6565,49 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quản lý người dùng: khoá / cảnh cáo</t>
+          <t xml:space="preserve">Tab Nhật ký admin (dùng adminlog.js đã có)</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KD09</t>
+          <t xml:space="preserve">CM02, KD11</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">auth.js, admin-users.js</t>
+          <t xml:space="preserve">admin-log.js</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">6 giờ</t>
+          <t xml:space="preserve">3 giờ</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">P2</t>
+          <t xml:space="preserve">P3</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tab Nhật ký admin (dùng adminlog.js đã có)</t>
+          <t xml:space="preserve">Trình dựng build + chia sẻ link + bình chọn Hữu ích</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">CM02, KD11</t>
+          <t xml:space="preserve">N02, N05, HD07, HD09</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin-log.js</t>
+          <t xml:space="preserve">build.js, build-detail.js</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 giờ</t>
+          <t xml:space="preserve">12 giờ</t>
         </is>
       </c>
     </row>
@@ -6354,22 +6619,22 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trình dựng build + chia sẻ link + bình chọn Hữu ích</t>
+          <t xml:space="preserve">Dark/Light mode</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">N02, N05, HD07, HD09</t>
+          <t xml:space="preserve">N03</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">build.js, build-detail.js</t>
+          <t xml:space="preserve">variables.css, layout.js</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">12 giờ</t>
+          <t xml:space="preserve">3 giờ</t>
         </is>
       </c>
     </row>
@@ -6381,22 +6646,22 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dark/Light mode</t>
+          <t xml:space="preserve">So sánh trang bị</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">N03</t>
+          <t xml:space="preserve">N04</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">variables.css, layout.js</t>
+          <t xml:space="preserve">compare.js</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 giờ</t>
+          <t xml:space="preserve">4 giờ</t>
         </is>
       </c>
     </row>
@@ -6408,22 +6673,22 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">So sánh trang bị</t>
+          <t xml:space="preserve">Biểu đồ radar chỉ số tướng</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">N04</t>
+          <t xml:space="preserve">N06</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">compare.js</t>
+          <t xml:space="preserve">hero-detail, compare</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 giờ</t>
+          <t xml:space="preserve">6 giờ</t>
         </is>
       </c>
     </row>
@@ -6435,22 +6700,22 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Biểu đồ radar chỉ số tướng</t>
+          <t xml:space="preserve">Xuất / nhập dữ liệu người dùng</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">N06</t>
+          <t xml:space="preserve">N07</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">hero-detail, compare</t>
+          <t xml:space="preserve">storage.js</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">6 giờ</t>
+          <t xml:space="preserve">3 giờ</t>
         </is>
       </c>
     </row>
@@ -6462,54 +6727,27 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Xuất / nhập dữ liệu người dùng</t>
+          <t xml:space="preserve">PWA + đa ngôn ngữ</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">N07</t>
+          <t xml:space="preserve">N10, N11</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">storage.js</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 giờ</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P3</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PWA + đa ngôn ngữ</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">N10, N11</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
           <t xml:space="preserve">16 giờ</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E20"/>
+  <autoFilter ref="A1:E19"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat(admin): duyet/tu choi bai o tab Cho duyet + test kiem duyet (KD03/KD12/CM06)
feed.js: them getPendingPosts(), approvePost(), rejectPost() (chi admin, ghi reviewedBy/reviewedAt + logAdminAction).

admin-pending.js: muc 'Bai viet cho duyet' voi nut Duyet/Tu choi + o ly do (tuy chon), cap nhat badge.

test-admin-pending.cjs (24 PASS) + test-admin-data.cjs (23 PASS, lop gop du lieu adminDataCheckRun/Load).

Cap nhat aov-hub-data.json + AOV_HUB.xlsx.
</commit_message>
<xml_diff>
--- a/AOV_HUB.xlsx
+++ b/AOV_HUB.xlsx
@@ -1373,8 +1373,89 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KD03</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sửa trạng thái</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Một phần -&gt; Đã xong</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">admin-pending.js: mục 'Bài viết chờ duyệt' + nút Duyệt/Từ chối kèm ô lý do (tuỳ chọn); approvePost()/rejectPost() trong feed.js (chỉ admin, ghi reviewedBy/reviewedAt + nhật ký); badge 'Chờ duyệt' tự cập nhật.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KD12 / CM06</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sửa trạng thái</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chưa làm / Một phần -&gt; Đã xong</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">test-admin-pending.cjs (24 PASS) kiểm duyệt; test-admin-data.cjs (23 PASS) lớp gộp dữ liệu (adminDataCheckRun/Load + loadData).</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Số liệu</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cập nhật</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Thêm admin-pending.js (JS top-level 25 -&gt; 26); test 17 -&gt; 19 file; 'Việc nên làm tiếp' P0 admin-pending -&gt; còn 7 file tab; npm test 18/19 PASS (test-feed-page đỏ do bài 'xcascsâccs' lúc chạy app trong posts.json, không liên quan).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E32"/>
+  <autoFilter ref="A1:E35"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -4252,14 +4333,14 @@
           <t xml:space="preserve">tools/</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Một phần</t>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã xong</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Có test-admin-shell, test-admin-page, test-hero-admin, test-datastore; chưa có test-admin-data/items/builds riêng.</t>
+          <t xml:space="preserve">test-admin-data.cjs: dữ liệu thật (32 tướng/40 trang bị/32 build) qua adminDataCheckRun() 0 lỗi; bắt được id trùng, heroId/trang bị/related hỏng; loadData() trả rỗng khi file thiếu/HTTP lỗi; adminDataCheckLoad() gom đủ items/builds/posts/users, 23 test PASS.</t>
         </is>
       </c>
     </row>
@@ -4345,17 +4426,17 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin.js, admin.html, feed.js</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Một phần</t>
+          <t xml:space="preserve">admin-pending.js, feed.js, admin.html</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã xong</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Khung đã có mục 'Chờ duyệt' + badge đếm bài pending; admin-pending.js chưa viết (hiện 'Mục này đang được phát triển.'); chưa có approvePost()/rejectPost().</t>
+          <t xml:space="preserve">admin-pending.js vẽ mục 'Bài viết chờ duyệt' với nút Duyệt/Từ chối + ô lý do (tuỳ chọn); approvePost()/rejectPost() (chỉ admin) đổi status, ghi reviewedBy/reviewedAt + logAdminAction; badge 'Chờ duyệt' tự cập nhật. test-admin-pending.cjs 24 test PASS.</t>
         </is>
       </c>
     </row>
@@ -4633,12 +4714,17 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">tools/test-moderation.cjs</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Chưa làm</t>
+          <t xml:space="preserve">tools/test-admin-pending.cjs</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã xong</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">test-admin-pending.cjs: getPendingPosts() (chỉ bài pending, mới nhất trước), render + escapeHtml, approvePost()/rejectPost() (có/không lý do, ghi nhật ký), chặn quyền user thường/khách, bấm nút DOM + cập nhật badge; 24 test PASS.</t>
         </is>
       </c>
     </row>
@@ -4990,7 +5076,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">test-hero-admin + test-admin-shell bao phủ tướng và khung; chưa có admin-items/builds.</t>
+          <t xml:space="preserve">test-hero-admin + test-admin-shell bao phủ tướng và khung; test-admin-data.cjs bổ sung lớp kiểm tra/gộp dữ liệu; chưa có admin-items/builds.</t>
         </is>
       </c>
     </row>
@@ -6295,49 +6381,49 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Viết 8 file tab admin còn thiếu để bỏ placeholder 'Mục này đang được phát triển.'</t>
+          <t xml:space="preserve">Viết 7 file tab admin còn thiếu để bỏ placeholder 'Mục này đang được phát triển.'</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">CM03, KD03, KD11, AD05-AD08</t>
+          <t xml:space="preserve">CM03, KD11, AD05-AD08</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/js/admin-pending/build-review/reports/users/items/builds/log/banned.js</t>
+          <t xml:space="preserve">src/js/admin-build-review/reports/users/items/builds/log/banned.js</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">16-24 giờ</t>
+          <t xml:space="preserve">14-21 giờ</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">P0</t>
+          <t xml:space="preserve">P1</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tab Chờ duyệt + approvePost()/rejectPost() (duyệt/từ chối kèm lý do) — nối vào mục 'Chờ duyệt' đã có</t>
+          <t xml:space="preserve">Thêm lane + title cho 32 tướng + select lọc đường đi</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KD03</t>
+          <t xml:space="preserve">L06</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/js/admin-pending.js, admin.js, feed.js</t>
+          <t xml:space="preserve">src/data/heroes.json, hero.js, hero-admin.js</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">8 giờ</t>
+          <t xml:space="preserve">4 giờ</t>
         </is>
       </c>
     </row>
@@ -6349,49 +6435,49 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Thêm lane + title cho 32 tướng + select lọc đường đi</t>
+          <t xml:space="preserve">Báo cáo vi phạm (aov_reports) + tab xử lý cho admin</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">L06</t>
+          <t xml:space="preserve">KD05, KD06</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/data/heroes.json, hero.js, hero-admin.js</t>
+          <t xml:space="preserve">feed.js, admin-reports.js</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 giờ</t>
+          <t xml:space="preserve">12 giờ</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">P1</t>
+          <t xml:space="preserve">P2</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Báo cáo vi phạm (aov_reports) + tab xử lý cho admin</t>
+          <t xml:space="preserve">Quản lý Trang bị (form thêm/sửa/xoá an toàn)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KD05, KD06</t>
+          <t xml:space="preserve">AD05, AD06</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">feed.js, admin-reports.js</t>
+          <t xml:space="preserve">admin-items.js</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">12 giờ</t>
+          <t xml:space="preserve">16 giờ</t>
         </is>
       </c>
     </row>
@@ -6403,22 +6489,22 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quản lý Trang bị (form thêm/sửa/xoá an toàn)</t>
+          <t xml:space="preserve">Quản lý Build + danh sách tướng thiếu build</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">AD05, AD06</t>
+          <t xml:space="preserve">AD07, AD08</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin-items.js</t>
+          <t xml:space="preserve">admin-builds.js</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">16 giờ</t>
+          <t xml:space="preserve">11 giờ</t>
         </is>
       </c>
     </row>
@@ -6430,22 +6516,22 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quản lý Build + danh sách tướng thiếu build</t>
+          <t xml:space="preserve">Trang chi tiết hướng dẫn build + mở rộng builds.json</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">AD07, AD08</t>
+          <t xml:space="preserve">HD01, HD02</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin-builds.js</t>
+          <t xml:space="preserve">build-detail.html/js, builds.json</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">11 giờ</t>
+          <t xml:space="preserve">13 giờ</t>
         </is>
       </c>
     </row>
@@ -6457,22 +6543,22 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trang chi tiết hướng dẫn build + mở rộng builds.json</t>
+          <t xml:space="preserve">Áp dụng bộ lọc từ khoá cấm vào nội dung</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HD01, HD02</t>
+          <t xml:space="preserve">KD07</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">build-detail.html/js, builds.json</t>
+          <t xml:space="preserve">feed.js, search.js</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">13 giờ</t>
+          <t xml:space="preserve">5 giờ</t>
         </is>
       </c>
     </row>
@@ -6484,17 +6570,17 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Áp dụng bộ lọc từ khoá cấm vào nội dung</t>
+          <t xml:space="preserve">Kiểm duyệt bình luận (trường hidden + UI admin)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KD07</t>
+          <t xml:space="preserve">KD08</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">feed.js, search.js</t>
+          <t xml:space="preserve">feed.js, admin.js</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -6511,22 +6597,22 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kiểm duyệt bình luận (trường hidden + UI admin)</t>
+          <t xml:space="preserve">Quản lý người dùng: khoá / cảnh cáo</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KD08</t>
+          <t xml:space="preserve">KD09</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">feed.js, admin.js</t>
+          <t xml:space="preserve">auth.js, admin-users.js</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">5 giờ</t>
+          <t xml:space="preserve">6 giờ</t>
         </is>
       </c>
     </row>
@@ -6538,49 +6624,49 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quản lý người dùng: khoá / cảnh cáo</t>
+          <t xml:space="preserve">Tab Nhật ký admin (dùng adminlog.js đã có)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KD09</t>
+          <t xml:space="preserve">CM02, KD11</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">auth.js, admin-users.js</t>
+          <t xml:space="preserve">admin-log.js</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">6 giờ</t>
+          <t xml:space="preserve">3 giờ</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">P2</t>
+          <t xml:space="preserve">P3</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tab Nhật ký admin (dùng adminlog.js đã có)</t>
+          <t xml:space="preserve">Trình dựng build + chia sẻ link + bình chọn Hữu ích</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">CM02, KD11</t>
+          <t xml:space="preserve">N02, N05, HD07, HD09</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin-log.js</t>
+          <t xml:space="preserve">build.js, build-detail.js</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 giờ</t>
+          <t xml:space="preserve">12 giờ</t>
         </is>
       </c>
     </row>
@@ -6592,22 +6678,22 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trình dựng build + chia sẻ link + bình chọn Hữu ích</t>
+          <t xml:space="preserve">Dark/Light mode</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">N02, N05, HD07, HD09</t>
+          <t xml:space="preserve">N03</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">build.js, build-detail.js</t>
+          <t xml:space="preserve">variables.css, layout.js</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">12 giờ</t>
+          <t xml:space="preserve">3 giờ</t>
         </is>
       </c>
     </row>
@@ -6619,22 +6705,22 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dark/Light mode</t>
+          <t xml:space="preserve">So sánh trang bị</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">N03</t>
+          <t xml:space="preserve">N04</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">variables.css, layout.js</t>
+          <t xml:space="preserve">compare.js</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 giờ</t>
+          <t xml:space="preserve">4 giờ</t>
         </is>
       </c>
     </row>
@@ -6646,22 +6732,22 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">So sánh trang bị</t>
+          <t xml:space="preserve">Biểu đồ radar chỉ số tướng</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">N04</t>
+          <t xml:space="preserve">N06</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">compare.js</t>
+          <t xml:space="preserve">hero-detail, compare</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 giờ</t>
+          <t xml:space="preserve">6 giờ</t>
         </is>
       </c>
     </row>
@@ -6673,22 +6759,22 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Biểu đồ radar chỉ số tướng</t>
+          <t xml:space="preserve">Xuất / nhập dữ liệu người dùng</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">N06</t>
+          <t xml:space="preserve">N07</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">hero-detail, compare</t>
+          <t xml:space="preserve">storage.js</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">6 giờ</t>
+          <t xml:space="preserve">3 giờ</t>
         </is>
       </c>
     </row>
@@ -6700,54 +6786,27 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Xuất / nhập dữ liệu người dùng</t>
+          <t xml:space="preserve">PWA + đa ngôn ngữ</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">N07</t>
+          <t xml:space="preserve">N10, N11</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">storage.js</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 giờ</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P3</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PWA + đa ngôn ngữ</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">N10, N11</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
           <t xml:space="preserve">16 giờ</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E19"/>
+  <autoFilter ref="A1:E18"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -7639,14 +7698,14 @@
           <t xml:space="preserve">Có</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Chưa làm</t>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã có</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KD03: mục 'Chờ duyệt' đã có trong khung nhưng chưa có approvePost()/rejectPost().</t>
+          <t xml:space="preserve">KD03: approvePost()/rejectPost() kiểm tra admin ở tầng dữ liệu; mục 'Bài viết chờ duyệt' có nút Duyệt/Từ chối + ô lý do.</t>
         </is>
       </c>
     </row>

</xml_diff>